<commit_message>
corrections SVM et surapprentissage
</commit_message>
<xml_diff>
--- a/models/model_comparison_recap_final.xlsx
+++ b/models/model_comparison_recap_final.xlsx
@@ -807,10 +807,10 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>0.61</v>
+        <v>0.59</v>
       </c>
       <c r="C23" t="n">
-        <v>0.63</v>
+        <v>0.66</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -868,7 +868,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>non disponible</t>
+          <t>oui (gap F1 train-val +0.22)</t>
         </is>
       </c>
     </row>
@@ -922,7 +922,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>non disponible</t>
+          <t>oui (gap F1 train-val +0.18)</t>
         </is>
       </c>
     </row>
@@ -940,7 +940,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>non disponible</t>
+          <t>oui (gap F1 train-val +0.17)</t>
         </is>
       </c>
     </row>
@@ -958,7 +958,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>non disponible</t>
+          <t>non (gap F1 train-val +0.00)</t>
         </is>
       </c>
     </row>
@@ -994,7 +994,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>non disponible</t>
+          <t>oui (gap F1 train-val +0.64)</t>
         </is>
       </c>
     </row>
@@ -1012,7 +1012,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>non disponible</t>
+          <t>oui (gap F1 train-val +0.42)</t>
         </is>
       </c>
     </row>
@@ -1030,7 +1030,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>non disponible</t>
+          <t>non (gap F1 train-val +0.02)</t>
         </is>
       </c>
     </row>
@@ -1048,7 +1048,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>non disponible</t>
+          <t>non applicable (aucun apprentissage)</t>
         </is>
       </c>
     </row>
@@ -1066,7 +1066,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>non disponible</t>
+          <t>non applicable (aucun apprentissage)</t>
         </is>
       </c>
     </row>

</xml_diff>